<commit_message>
fix: validaciones para carga masiva
</commit_message>
<xml_diff>
--- a/frontend/public/template_animales.xlsx
+++ b/frontend/public/template_animales.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>IdCaravana</t>
   </si>
@@ -50,16 +50,16 @@
     <t>Toro</t>
   </si>
   <si>
-    <t/>
+    <t>2022-08-03</t>
   </si>
   <si>
     <t>Hereford</t>
   </si>
   <si>
-    <t>Lote Principal</t>
+    <t>789</t>
   </si>
   <si>
-    <t>Lola</t>
+    <t>2024-02-20</t>
   </si>
 </sst>
 </file>
@@ -67,13 +67,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
     </font>
   </fonts>
   <fills count="2">
@@ -96,8 +101,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -106,73 +113,76 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" style="1" width="18.0" customWidth="true"/>
+    <col min="2" max="2" style="1" width="18.0" customWidth="true"/>
+    <col min="3" max="3" style="1" width="18.0" customWidth="true"/>
+    <col min="4" max="4" style="1" width="18.0" customWidth="true"/>
+    <col min="5" max="5" style="1" width="18.0" customWidth="true"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="0">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="0">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s" s="0">
+      <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="0">
+      <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E3" t="s" s="0">
-        <v>14</v>
+      <c r="E3" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>12</v>
+      <c r="A4" s="1" t="s">
+        <v>14</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C4" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>12</v>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: Campo sensor en carga de animales
Se agrega el campo sensor opcional en la carga masiva de animales
</commit_message>
<xml_diff>
--- a/frontend/public/template_animales.xlsx
+++ b/frontend/public/template_animales.xlsx
@@ -12,18 +12,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>IdCaravana</t>
   </si>
   <si>
-    <t>Alias</t>
+    <t>Alias (opcional)</t>
   </si>
   <si>
     <t>FechaNacimiento</t>
   </si>
   <si>
-    <t>Raza</t>
+    <t>Raza (opcional)</t>
   </si>
   <si>
     <t>RodeoLote</t>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>2024-02-20</t>
+  </si>
+  <si>
+    <t>Sensor (opcional)</t>
+  </si>
+  <si>
+    <t>A84041C2F1B3D001</t>
   </si>
 </sst>
 </file>
@@ -111,7 +117,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" style="1" width="18.0" customWidth="true"/>
@@ -119,6 +125,7 @@
     <col min="3" max="3" style="1" width="18.0" customWidth="true"/>
     <col min="4" max="4" style="1" width="18.0" customWidth="true"/>
     <col min="5" max="5" style="1" width="18.0" customWidth="true"/>
+    <col min="6" max="6" style="1" width="22.0" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -137,6 +144,9 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="2" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
@@ -154,6 +164,9 @@
       <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="F2" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
@@ -171,6 +184,7 @@
       <c r="E3" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="F3" s="1"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
@@ -184,6 +198,7 @@
       <c r="E4" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="F4" s="1"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>